<commit_message>
included b10br kb x b10br kd as well - changed the colours and legend lables to ensure clarity
this will basically be the last comparison one
change with levenshtein 0

revisit soon with varying levenshtein thresholds
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/pc_summary_statistics.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/pc_summary_statistics.xlsx
@@ -894,16 +894,16 @@
         <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0006537254146487813</v>
+        <v>0.0007741148578617333</v>
       </c>
       <c r="G9" t="n">
-        <v>4.274722143060701e-05</v>
+        <v>4.327457677400295e-05</v>
       </c>
       <c r="H9" t="n">
-        <v>0.002063287283014385</v>
+        <v>0.002391362923702407</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -912,19 +912,19 @@
         <v>0.01373626373626374</v>
       </c>
       <c r="K9" t="n">
-        <v>0.009239311767858078</v>
+        <v>0.01094081453106472</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0.009x</t>
+          <t>0.011x</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>0.009239311767858078</v>
+        <v>0.01094081453106472</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.009x</t>
+          <t>0.011x</t>
         </is>
       </c>
     </row>
@@ -966,11 +966,11 @@
         <v>0.01373626373626374</v>
       </c>
       <c r="K10" t="n">
-        <v>0.4668610498814553</v>
+        <v>0.3942553618724525</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0.467x</t>
+          <t>0.394x</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1538,16 +1538,16 @@
         <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="F21" t="n">
-        <v>0.005018058172008242</v>
+        <v>0.00712907591715185</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0007971901934052731</v>
+        <v>0.001094615536981008</v>
       </c>
       <c r="H21" t="n">
-        <v>0.01467312890150336</v>
+        <v>0.01887715056742475</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -1556,19 +1556,19 @@
         <v>0.1025641025641026</v>
       </c>
       <c r="K21" t="n">
-        <v>0.05858732315556182</v>
+        <v>0.08323408383118734</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0.059x</t>
+          <t>0.083x</t>
         </is>
       </c>
       <c r="M21" t="n">
-        <v>0.05858732315556182</v>
+        <v>0.08323408383118734</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.059x</t>
+          <t>0.083x</t>
         </is>
       </c>
     </row>
@@ -1610,11 +1610,11 @@
         <v>0.1025641025641026</v>
       </c>
       <c r="K22" t="n">
-        <v>0.4813456474062321</v>
+        <v>0.3388125596637537</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0.481x</t>
+          <t>0.339x</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -2182,16 +2182,16 @@
         <v>2</v>
       </c>
       <c r="E33" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="F33" t="n">
-        <v>0.004972153294705976</v>
+        <v>0.004776063527785849</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0004711737886845994</v>
+        <v>0.0004292298818519529</v>
       </c>
       <c r="H33" t="n">
-        <v>0.01235829636093292</v>
+        <v>0.01440360389873472</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -2200,19 +2200,19 @@
         <v>0.06818181818181818</v>
       </c>
       <c r="K33" t="n">
-        <v>0.05705587741330239</v>
+        <v>0.05480573083891778</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0.057x</t>
+          <t>0.055x</t>
         </is>
       </c>
       <c r="M33" t="n">
-        <v>0.05705587741330239</v>
+        <v>0.05480573083891778</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>0.057x</t>
+          <t>0.055x</t>
         </is>
       </c>
     </row>
@@ -2254,11 +2254,11 @@
         <v>0.06818181818181818</v>
       </c>
       <c r="K34" t="n">
-        <v>0.6731772714654718</v>
+        <v>0.7008157594147281</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0.673x</t>
+          <t>0.701x</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2826,16 +2826,16 @@
         <v>2</v>
       </c>
       <c r="E45" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="F45" t="n">
-        <v>0.0004167374584717313</v>
+        <v>0.0005932209720691081</v>
       </c>
       <c r="G45" t="n">
-        <v>1.885333986915782e-05</v>
+        <v>4.67032399052543e-06</v>
       </c>
       <c r="H45" t="n">
-        <v>0.001699422409607001</v>
+        <v>0.002223799704063026</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
@@ -2844,19 +2844,19 @@
         <v>0.01316391941391941</v>
       </c>
       <c r="K45" t="n">
-        <v>0.005941837624734539</v>
+        <v>0.008458137419535383</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0.006x</t>
+          <t>0.008x</t>
         </is>
       </c>
       <c r="M45" t="n">
-        <v>0.005941837624734539</v>
+        <v>0.008458137419535383</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>0.006x</t>
+          <t>0.008x</t>
         </is>
       </c>
     </row>
@@ -2898,11 +2898,11 @@
         <v>0.01316391941391941</v>
       </c>
       <c r="K46" t="n">
-        <v>0.4666666666666667</v>
+        <v>0.3278331174668676</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>0.467x</t>
+          <t>0.328x</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3470,16 +3470,16 @@
         <v>2</v>
       </c>
       <c r="E57" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="F57" t="n">
-        <v>0.002177832778921493</v>
+        <v>0.003686440837408867</v>
       </c>
       <c r="G57" t="n">
-        <v>8.529722014482592e-05</v>
+        <v>0.000206419994879848</v>
       </c>
       <c r="H57" t="n">
-        <v>0.01016949922012155</v>
+        <v>0.01332872434129193</v>
       </c>
       <c r="I57" t="n">
         <v>0</v>
@@ -3488,19 +3488,19 @@
         <v>0.07869142351900972</v>
       </c>
       <c r="K57" t="n">
-        <v>0.02618622821125659</v>
+        <v>0.04432570856220192</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>0.026x</t>
+          <t>0.044x</t>
         </is>
       </c>
       <c r="M57" t="n">
-        <v>0.02618622821125659</v>
+        <v>0.04432570856220192</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>0.026x</t>
+          <t>0.044x</t>
         </is>
       </c>
     </row>
@@ -3542,11 +3542,11 @@
         <v>0.07869142351900972</v>
       </c>
       <c r="K58" t="n">
-        <v>0.4714861649135916</v>
+        <v>0.2785391303006877</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>0.471x</t>
+          <t>0.279x</t>
         </is>
       </c>
       <c r="M58" t="n">
@@ -4114,16 +4114,16 @@
         <v>2</v>
       </c>
       <c r="E69" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="F69" t="n">
-        <v>0.001864180241102332</v>
+        <v>0.00315228236576409</v>
       </c>
       <c r="G69" t="n">
-        <v>5.678889812611355e-05</v>
+        <v>0.000302155638177779</v>
       </c>
       <c r="H69" t="n">
-        <v>0.008826823132653219</v>
+        <v>0.01157355516675025</v>
       </c>
       <c r="I69" t="n">
         <v>0</v>
@@ -4132,19 +4132,19 @@
         <v>0.06818181818181818</v>
       </c>
       <c r="K69" t="n">
-        <v>0.02147929010255906</v>
+        <v>0.03632094468472122</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>0.021x</t>
+          <t>0.036x</t>
         </is>
       </c>
       <c r="M69" t="n">
-        <v>0.02147929010255906</v>
+        <v>0.03632094468472122</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>0.021x</t>
+          <t>0.036x</t>
         </is>
       </c>
     </row>
@@ -4186,11 +4186,11 @@
         <v>0.06818181818181818</v>
       </c>
       <c r="K70" t="n">
-        <v>0.6953361567632769</v>
+        <v>0.4112042558243152</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>0.695x</t>
+          <t>0.411x</t>
         </is>
       </c>
       <c r="M70" t="n">

</xml_diff>

<commit_message>
Added heatmaps for just Kb and just Kd separaetly
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/pc_summary_statistics.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/pc_summary_statistics.xlsx
@@ -825,12 +825,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CDR3</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -845,19 +845,19 @@
         <v>27</v>
       </c>
       <c r="F8" t="n">
-        <v>0.070754773848305</v>
+        <v>0.1535210569854885</v>
       </c>
       <c r="G8" t="n">
-        <v>0.02436966427305397</v>
+        <v>0.1377995642701525</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1390515058616148</v>
+        <v>0.09476668652678683</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0008048289738430583</v>
+        <v>0.02998084291187739</v>
       </c>
       <c r="J8" t="n">
-        <v>0.6783511846802986</v>
+        <v>0.399400299850075</v>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
@@ -877,12 +877,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CDR3</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -894,49 +894,49 @@
         <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0007741148578617333</v>
+        <v>0.02973927276910436</v>
       </c>
       <c r="G9" t="n">
-        <v>4.327457677400295e-05</v>
+        <v>0.01002731165898068</v>
       </c>
       <c r="H9" t="n">
-        <v>0.002391362923702407</v>
+        <v>0.04311019545593976</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.01373626373626374</v>
+        <v>0.1730523627075351</v>
       </c>
       <c r="K9" t="n">
-        <v>0.01094081453106472</v>
+        <v>0.1937146170894032</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0.011x</t>
+          <t>0.194x</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>0.01094081453106472</v>
+        <v>0.1937146170894032</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.011x</t>
+          <t>0.194x</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CDR3</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -948,49 +948,49 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0003051989334171198</v>
+        <v>0.01590863184638534</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>0.002576995068464651</v>
       </c>
       <c r="H10" t="n">
-        <v>0.001441114284775114</v>
+        <v>0.03346028052793922</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0.01373626373626374</v>
+        <v>0.1730523627075351</v>
       </c>
       <c r="K10" t="n">
-        <v>0.3942553618724525</v>
+        <v>0.534936814692811</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0.394x</t>
+          <t>0.535x</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>0.004313474792124307</v>
+        <v>0.1036250802252429</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.004x</t>
+          <t>0.104x</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CDR3</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1002,49 +1002,49 @@
         <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0003679439371722536</v>
+        <v>0.01117642533837137</v>
       </c>
       <c r="G11" t="n">
-        <v>1.71860818924986e-05</v>
+        <v>0.001479289940828402</v>
       </c>
       <c r="H11" t="n">
-        <v>0.001476555200658624</v>
+        <v>0.02654862015613111</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0.01373626373626374</v>
+        <v>0.1730523627075351</v>
       </c>
       <c r="K11" t="n">
-        <v>1.205587231425148</v>
+        <v>0.7025384361327592</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1.206x</t>
+          <t>0.703x</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>0.00520027013245931</v>
+        <v>0.07280060180557386</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0.005x</t>
+          <t>0.073x</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CDR3</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1059,46 +1059,46 @@
         <v>351</v>
       </c>
       <c r="F12" t="n">
-        <v>0.000179303612948414</v>
+        <v>0.006562829681891059</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>0.0004801920768307323</v>
       </c>
       <c r="H12" t="n">
-        <v>0.001045401853743629</v>
+        <v>0.02015358805975859</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0.01373626373626374</v>
+        <v>0.1730523627075351</v>
       </c>
       <c r="K12" t="n">
-        <v>0.4873123180841344</v>
+        <v>0.5872029278770629</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0.487x</t>
+          <t>0.587x</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>0.002534155692912435</v>
+        <v>0.04274872653144517</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.003x</t>
+          <t>0.043x</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CDR3</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1113,34 +1113,34 @@
         <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>3.112614202830989e-08</v>
+        <v>0.0001169694818177544</v>
       </c>
       <c r="G13" t="n">
-        <v>3.112614202830989e-08</v>
+        <v>0.0001169694818177544</v>
       </c>
       <c r="H13" t="n">
-        <v>9.78051048024283e-09</v>
+        <v>7.787060743328694e-05</v>
       </c>
       <c r="I13" t="n">
-        <v>2.421027674426409e-08</v>
+        <v>6.190664724656162e-05</v>
       </c>
       <c r="J13" t="n">
-        <v>3.804200731235569e-08</v>
+        <v>0.0001720323163889472</v>
       </c>
       <c r="K13" t="n">
-        <v>0.0001735946170658866</v>
+        <v>0.01782302565926867</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0.000x</t>
+          <t>0.018x</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>4.399157870964709e-07</v>
+        <v>0.0007619116498710066</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0.000x</t>
+          <t>0.001x</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1167,19 +1167,19 @@
         <v>27</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1535210569854885</v>
+        <v>0.1543594252699805</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1377995642701525</v>
+        <v>0.1158402203856749</v>
       </c>
       <c r="H14" t="n">
-        <v>0.09476668652678683</v>
+        <v>0.1053118123752471</v>
       </c>
       <c r="I14" t="n">
-        <v>0.02998084291187739</v>
+        <v>0.01696020874103066</v>
       </c>
       <c r="J14" t="n">
-        <v>0.399400299850075</v>
+        <v>0.4321200621010868</v>
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1219,34 +1219,34 @@
         <v>54</v>
       </c>
       <c r="F15" t="n">
-        <v>0.02973927276910436</v>
+        <v>0.01799049604619476</v>
       </c>
       <c r="G15" t="n">
-        <v>0.01002731165898068</v>
+        <v>0.006699632021885506</v>
       </c>
       <c r="H15" t="n">
-        <v>0.04311019545593976</v>
+        <v>0.04923130678847103</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1730523627075351</v>
+        <v>0.3612068965517241</v>
       </c>
       <c r="K15" t="n">
-        <v>0.1937146170894032</v>
+        <v>0.1165493847539838</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0.194x</t>
+          <t>0.117x</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>0.1937146170894032</v>
+        <v>0.1165493847539838</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.194x</t>
+          <t>0.117x</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1273,34 +1273,34 @@
         <v>108</v>
       </c>
       <c r="F16" t="n">
-        <v>0.01590863184638534</v>
+        <v>0.0126945918964665</v>
       </c>
       <c r="G16" t="n">
-        <v>0.002576995068464651</v>
+        <v>0.00271411335360849</v>
       </c>
       <c r="H16" t="n">
-        <v>0.03346028052793922</v>
+        <v>0.04209634359971922</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0.1730523627075351</v>
+        <v>0.3612068965517241</v>
       </c>
       <c r="K16" t="n">
-        <v>0.534936814692811</v>
+        <v>0.7056276749607234</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0.535x</t>
+          <t>0.706x</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>0.1036250802252429</v>
+        <v>0.08224047138205635</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>0.104x</t>
+          <t>0.082x</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1327,34 +1327,34 @@
         <v>189</v>
       </c>
       <c r="F17" t="n">
-        <v>0.01117642533837137</v>
+        <v>0.007167034355277721</v>
       </c>
       <c r="G17" t="n">
-        <v>0.001479289940828402</v>
+        <v>0.0004973474801061008</v>
       </c>
       <c r="H17" t="n">
-        <v>0.02654862015613111</v>
+        <v>0.02799023559308392</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0.1730523627075351</v>
+        <v>0.3612068965517241</v>
       </c>
       <c r="K17" t="n">
-        <v>0.7025384361327592</v>
+        <v>0.5645738290549256</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0.703x</t>
+          <t>0.565x</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>0.07280060180557386</v>
+        <v>0.04643081783144958</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.073x</t>
+          <t>0.046x</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1381,34 +1381,34 @@
         <v>351</v>
       </c>
       <c r="F18" t="n">
-        <v>0.006562829681891059</v>
+        <v>0.005554557126008002</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0004801920768307323</v>
+        <v>0.0002658631690889755</v>
       </c>
       <c r="H18" t="n">
-        <v>0.02015358805975859</v>
+        <v>0.02456813708969558</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0.1730523627075351</v>
+        <v>0.3612068965517241</v>
       </c>
       <c r="K18" t="n">
-        <v>0.5872029278770629</v>
+        <v>0.7750147202681804</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.587x</t>
+          <t>0.775x</t>
         </is>
       </c>
       <c r="M18" t="n">
-        <v>0.04274872653144517</v>
+        <v>0.03598456729346375</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>0.043x</t>
+          <t>0.036x</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1435,46 +1435,46 @@
         <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0001169694818177544</v>
+        <v>1.507953647152783e-05</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0001169694818177544</v>
+        <v>1.507953647152783e-05</v>
       </c>
       <c r="H19" t="n">
-        <v>7.787060743328694e-05</v>
+        <v>2.739550852279648e-06</v>
       </c>
       <c r="I19" t="n">
-        <v>6.190664724656162e-05</v>
+        <v>1.314238148647551e-05</v>
       </c>
       <c r="J19" t="n">
-        <v>0.0001720323163889472</v>
+        <v>1.701669145658016e-05</v>
       </c>
       <c r="K19" t="n">
-        <v>0.01782302565926867</v>
+        <v>0.00271480446225338</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.018x</t>
+          <t>0.003x</t>
         </is>
       </c>
       <c r="M19" t="n">
-        <v>0.0007619116498710066</v>
+        <v>9.769106386055242e-05</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0.001x</t>
+          <t>0.000x</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>FullAlpha</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1489,19 +1489,19 @@
         <v>27</v>
       </c>
       <c r="F20" t="n">
-        <v>0.08565092074072454</v>
+        <v>0.1428016801844224</v>
       </c>
       <c r="G20" t="n">
-        <v>0.03130113835245316</v>
+        <v>0.1301775147928994</v>
       </c>
       <c r="H20" t="n">
-        <v>0.160737741723825</v>
+        <v>0.09170777419687813</v>
       </c>
       <c r="I20" t="n">
-        <v>0.002012072434607646</v>
+        <v>0.0264367816091954</v>
       </c>
       <c r="J20" t="n">
-        <v>0.7838364167478091</v>
+        <v>0.3883058470764618</v>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
@@ -1521,12 +1521,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>FullAlpha</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1538,49 +1538,49 @@
         <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="F21" t="n">
-        <v>0.00712907591715185</v>
+        <v>0.01685383548180843</v>
       </c>
       <c r="G21" t="n">
-        <v>0.001094615536981008</v>
+        <v>0.005390588934741554</v>
       </c>
       <c r="H21" t="n">
-        <v>0.01887715056742475</v>
+        <v>0.02684572963874532</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0.1025641025641026</v>
+        <v>0.1298374481398354</v>
       </c>
       <c r="K21" t="n">
-        <v>0.08323408383118734</v>
+        <v>0.118022669341442</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0.083x</t>
+          <t>0.118x</t>
         </is>
       </c>
       <c r="M21" t="n">
-        <v>0.08323408383118734</v>
+        <v>0.118022669341442</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.083x</t>
+          <t>0.118x</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>FullAlpha</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1592,49 +1592,49 @@
         <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="F22" t="n">
-        <v>0.002415420459527441</v>
+        <v>0.008934128277050243</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0001757385769924955</v>
+        <v>0.001218086055301858</v>
       </c>
       <c r="H22" t="n">
-        <v>0.01027701012555062</v>
+        <v>0.02053450368074804</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0.1025641025641026</v>
+        <v>0.1298374481398354</v>
       </c>
       <c r="K22" t="n">
-        <v>0.3388125596637537</v>
+        <v>0.5300946651991172</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0.339x</t>
+          <t>0.530x</t>
         </is>
       </c>
       <c r="M22" t="n">
-        <v>0.02820075299411205</v>
+        <v>0.0625631873904578</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>0.028x</t>
+          <t>0.063x</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>FullAlpha</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1646,49 +1646,49 @@
         <v>4</v>
       </c>
       <c r="E23" t="n">
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="F23" t="n">
-        <v>0.002693106987006515</v>
+        <v>0.006610525272294024</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0004018576933695114</v>
+        <v>0.0009613073780341264</v>
       </c>
       <c r="H23" t="n">
-        <v>0.009552684334011262</v>
+        <v>0.0164585619713131</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0.1025641025641026</v>
+        <v>0.1298374481398354</v>
       </c>
       <c r="K23" t="n">
-        <v>1.11496405372562</v>
+        <v>0.7399183297238937</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.115x</t>
+          <t>0.740x</t>
         </is>
       </c>
       <c r="M23" t="n">
-        <v>0.03144282587643008</v>
+        <v>0.0462916491161505</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>0.031x</t>
+          <t>0.046x</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>FullAlpha</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1703,46 +1703,46 @@
         <v>351</v>
       </c>
       <c r="F24" t="n">
-        <v>0.001357784231723905</v>
+        <v>0.003841069855168812</v>
       </c>
       <c r="G24" t="n">
-        <v>0.0001018507740658829</v>
+        <v>0.0001560695445890689</v>
       </c>
       <c r="H24" t="n">
-        <v>0.006784993903677931</v>
+        <v>0.01245847079403397</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0.1025641025641026</v>
+        <v>0.1298374481398354</v>
       </c>
       <c r="K24" t="n">
-        <v>0.5041701790069361</v>
+        <v>0.5810536526147886</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0.504x</t>
+          <t>0.581x</t>
         </is>
       </c>
       <c r="M24" t="n">
-        <v>0.01585253515060368</v>
+        <v>0.0268979318045014</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>0.016x</t>
+          <t>0.027x</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CDR3a</t>
+          <t>FullAlpha</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1757,34 +1757,34 @@
         <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0001298955201225842</v>
+        <v>2.452959985183437e-05</v>
       </c>
       <c r="G25" t="n">
-        <v>0.0001298955201225842</v>
+        <v>2.452959985183437e-05</v>
       </c>
       <c r="H25" t="n">
-        <v>5.959042875484255e-05</v>
+        <v>1.282136692836654e-05</v>
       </c>
       <c r="I25" t="n">
-        <v>8.775872385622115e-05</v>
+        <v>1.546352435270545e-05</v>
       </c>
       <c r="J25" t="n">
-        <v>0.0001720323163889472</v>
+        <v>3.359567535096329e-05</v>
       </c>
       <c r="K25" t="n">
-        <v>0.09566727694109604</v>
+        <v>0.006386137398367183</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0.096x</t>
+          <t>0.006x</t>
         </is>
       </c>
       <c r="M25" t="n">
-        <v>0.001516568870471261</v>
+        <v>0.0001717738882354564</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>0.002x</t>
+          <t>0.000x</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullBeta</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1811,16 +1811,16 @@
         <v>27</v>
       </c>
       <c r="F26" t="n">
-        <v>0.1543594252699805</v>
+        <v>0.1540154431948367</v>
       </c>
       <c r="G26" t="n">
         <v>0.1158402203856749</v>
       </c>
       <c r="H26" t="n">
-        <v>0.1053118123752471</v>
+        <v>0.1055437468616878</v>
       </c>
       <c r="I26" t="n">
-        <v>0.01696020874103066</v>
+        <v>0.01686702078091511</v>
       </c>
       <c r="J26" t="n">
         <v>0.4321200621010868</v>
@@ -1848,7 +1848,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullBeta</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1863,13 +1863,13 @@
         <v>54</v>
       </c>
       <c r="F27" t="n">
-        <v>0.01799049604619476</v>
+        <v>0.01782030571915158</v>
       </c>
       <c r="G27" t="n">
-        <v>0.006699632021885506</v>
+        <v>0.006677088898509607</v>
       </c>
       <c r="H27" t="n">
-        <v>0.04923130678847103</v>
+        <v>0.04924877471640624</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -1878,19 +1878,19 @@
         <v>0.3612068965517241</v>
       </c>
       <c r="K27" t="n">
-        <v>0.1165493847539838</v>
+        <v>0.1157046679832493</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0.117x</t>
+          <t>0.116x</t>
         </is>
       </c>
       <c r="M27" t="n">
-        <v>0.1165493847539838</v>
+        <v>0.1157046679832493</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>0.117x</t>
+          <t>0.116x</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullBeta</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1917,13 +1917,13 @@
         <v>108</v>
       </c>
       <c r="F28" t="n">
-        <v>0.0126945918964665</v>
+        <v>0.01253593281963678</v>
       </c>
       <c r="G28" t="n">
         <v>0.00271411335360849</v>
       </c>
       <c r="H28" t="n">
-        <v>0.04209634359971922</v>
+        <v>0.04210089482392654</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -1932,19 +1932,19 @@
         <v>0.3612068965517241</v>
       </c>
       <c r="K28" t="n">
-        <v>0.7056276749607234</v>
+        <v>0.7034633982830242</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0.706x</t>
+          <t>0.703x</t>
         </is>
       </c>
       <c r="M28" t="n">
-        <v>0.08224047138205635</v>
+        <v>0.0813939989367056</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>0.082x</t>
+          <t>0.081x</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullBeta</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1971,13 +1971,13 @@
         <v>189</v>
       </c>
       <c r="F29" t="n">
-        <v>0.007167034355277721</v>
+        <v>0.00705422976093418</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0004973474801061008</v>
+        <v>0.0004251700680272109</v>
       </c>
       <c r="H29" t="n">
-        <v>0.02799023559308392</v>
+        <v>0.02797947491014535</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -1986,15 +1986,15 @@
         <v>0.3612068965517241</v>
       </c>
       <c r="K29" t="n">
-        <v>0.5645738290549256</v>
+        <v>0.5627207693618265</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0.565x</t>
+          <t>0.563x</t>
         </is>
       </c>
       <c r="M29" t="n">
-        <v>0.04643081783144958</v>
+        <v>0.04580209370309865</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullBeta</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2025,13 +2025,13 @@
         <v>351</v>
       </c>
       <c r="F30" t="n">
-        <v>0.005554557126008002</v>
+        <v>0.005335151368539006</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0002658631690889755</v>
+        <v>0.0002297794117647059</v>
       </c>
       <c r="H30" t="n">
-        <v>0.02456813708969558</v>
+        <v>0.02449839159150042</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -2040,19 +2040,19 @@
         <v>0.3612068965517241</v>
       </c>
       <c r="K30" t="n">
-        <v>0.7750147202681804</v>
+        <v>0.7563053018324826</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0.775x</t>
+          <t>0.756x</t>
         </is>
       </c>
       <c r="M30" t="n">
-        <v>0.03598456729346375</v>
+        <v>0.03464036630268168</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>0.036x</t>
+          <t>0.035x</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullBeta</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2079,30 +2079,30 @@
         <v>2</v>
       </c>
       <c r="F31" t="n">
-        <v>1.507953647152783e-05</v>
+        <v>8.290285626479562e-06</v>
       </c>
       <c r="G31" t="n">
-        <v>1.507953647152783e-05</v>
+        <v>8.290285626479562e-06</v>
       </c>
       <c r="H31" t="n">
-        <v>2.739550852279648e-06</v>
+        <v>1.770770382762725e-06</v>
       </c>
       <c r="I31" t="n">
-        <v>1.314238148647551e-05</v>
+        <v>7.038161880903741e-06</v>
       </c>
       <c r="J31" t="n">
-        <v>1.701669145658016e-05</v>
+        <v>9.542409372055383e-06</v>
       </c>
       <c r="K31" t="n">
-        <v>0.00271480446225338</v>
+        <v>0.001553898859433823</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0.003x</t>
+          <t>0.002x</t>
         </is>
       </c>
       <c r="M31" t="n">
-        <v>9.769106386055242e-05</v>
+        <v>5.382762568810689e-05</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -2113,12 +2113,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2133,19 +2133,19 @@
         <v>27</v>
       </c>
       <c r="F32" t="n">
-        <v>0.08714533050974928</v>
+        <v>0.1189728184806998</v>
       </c>
       <c r="G32" t="n">
-        <v>0.03391075472853033</v>
+        <v>0.09889502762430939</v>
       </c>
       <c r="H32" t="n">
-        <v>0.1486791053449375</v>
+        <v>0.08783902582119305</v>
       </c>
       <c r="I32" t="n">
-        <v>0.0008048289738430583</v>
+        <v>0.01463050973814183</v>
       </c>
       <c r="J32" t="n">
-        <v>0.6994482310938007</v>
+        <v>0.3754122938530735</v>
       </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
@@ -2165,12 +2165,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2182,49 +2182,49 @@
         <v>2</v>
       </c>
       <c r="E33" t="n">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="F33" t="n">
-        <v>0.004776063527785849</v>
+        <v>0.002964521997024178</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0004292298818519529</v>
+        <v>0.0006031249374148842</v>
       </c>
       <c r="H33" t="n">
-        <v>0.01440360389873472</v>
+        <v>0.005008898523871809</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>0.06818181818181818</v>
+        <v>0.02492163009404389</v>
       </c>
       <c r="K33" t="n">
-        <v>0.05480573083891778</v>
+        <v>0.02491764114594876</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0.055x</t>
+          <t>0.025x</t>
         </is>
       </c>
       <c r="M33" t="n">
-        <v>0.05480573083891778</v>
+        <v>0.02491764114594876</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>0.055x</t>
+          <t>0.025x</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2236,49 +2236,49 @@
         <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="F34" t="n">
-        <v>0.003347140588238225</v>
+        <v>0.001538019735305308</v>
       </c>
       <c r="G34" t="n">
-        <v>0.0002648893113267449</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0.009228045923148144</v>
+        <v>0.003843021418339992</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0.06818181818181818</v>
+        <v>0.02492163009404389</v>
       </c>
       <c r="K34" t="n">
-        <v>0.7008157594147281</v>
+        <v>0.5188086770309651</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0.701x</t>
+          <t>0.519x</t>
         </is>
       </c>
       <c r="M34" t="n">
-        <v>0.03840871987815535</v>
+        <v>0.01292748843766202</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>0.038x</t>
+          <t>0.013x</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2290,49 +2290,49 @@
         <v>4</v>
       </c>
       <c r="E35" t="n">
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="F35" t="n">
-        <v>0.002334549589353883</v>
+        <v>0.001486461098652004</v>
       </c>
       <c r="G35" t="n">
-        <v>0.000230859637340497</v>
+        <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>0.007912764679275474</v>
+        <v>0.004135700372420237</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>0.06818181818181818</v>
+        <v>0.02492163009404389</v>
       </c>
       <c r="K35" t="n">
-        <v>0.6974758089210346</v>
+        <v>0.9664772593811553</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0.697x</t>
+          <t>0.966x</t>
         </is>
       </c>
       <c r="M35" t="n">
-        <v>0.02678915296663782</v>
+        <v>0.01249412359591316</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>0.027x</t>
+          <t>0.012x</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2347,46 +2347,46 @@
         <v>351</v>
       </c>
       <c r="F36" t="n">
-        <v>0.001563182077865423</v>
+        <v>0.0008175586644413006</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0001166393293238564</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>0.006004885927801725</v>
+        <v>0.003130494385334906</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>0.06818181818181818</v>
+        <v>0.02492163009404389</v>
       </c>
       <c r="K36" t="n">
-        <v>0.669586152718244</v>
+        <v>0.5500034041810464</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0.670x</t>
+          <t>0.550x</t>
         </is>
       </c>
       <c r="M36" t="n">
-        <v>0.01793764586951155</v>
+        <v>0.006871810510010975</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>0.018x</t>
+          <t>0.007x</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Kd</t>
+          <t>Kb</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CDR3b</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2401,30 +2401,30 @@
         <v>2</v>
       </c>
       <c r="F37" t="n">
-        <v>1.584501002217626e-05</v>
+        <v>1.825348372995303e-08</v>
       </c>
       <c r="G37" t="n">
-        <v>1.584501002217626e-05</v>
+        <v>1.825348372995303e-08</v>
       </c>
       <c r="H37" t="n">
-        <v>1.657007775314753e-06</v>
+        <v>7.708653197898958e-10</v>
       </c>
       <c r="I37" t="n">
-        <v>1.467332858777236e-05</v>
+        <v>1.770839963494805e-08</v>
       </c>
       <c r="J37" t="n">
-        <v>1.701669145658016e-05</v>
+        <v>1.8798567824958e-08</v>
       </c>
       <c r="K37" t="n">
-        <v>0.0101363815812251</v>
+        <v>2.232681827478032e-05</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0.010x</t>
+          <t>0.000x</t>
         </is>
       </c>
       <c r="M37" t="n">
-        <v>0.0001818228232022554</v>
+        <v>1.534256644757405e-07</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -2435,12 +2435,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2455,19 +2455,19 @@
         <v>27</v>
       </c>
       <c r="F38" t="n">
-        <v>0.1189728184806998</v>
+        <v>0.070754773848305</v>
       </c>
       <c r="G38" t="n">
-        <v>0.09889502762430939</v>
+        <v>0.02436966427305397</v>
       </c>
       <c r="H38" t="n">
-        <v>0.08783902582119305</v>
+        <v>0.1390515058616148</v>
       </c>
       <c r="I38" t="n">
-        <v>0.01463050973814183</v>
+        <v>0.0008048289738430583</v>
       </c>
       <c r="J38" t="n">
-        <v>0.3754122938530735</v>
+        <v>0.6783511846802986</v>
       </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
@@ -2487,12 +2487,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2504,49 +2504,49 @@
         <v>2</v>
       </c>
       <c r="E39" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="F39" t="n">
-        <v>0.002964521997024178</v>
+        <v>0.0007741148578617333</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0006031249374148842</v>
+        <v>4.327457677400295e-05</v>
       </c>
       <c r="H39" t="n">
-        <v>0.005008898523871809</v>
+        <v>0.002391362923702407</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>0.02492163009404389</v>
+        <v>0.01373626373626374</v>
       </c>
       <c r="K39" t="n">
-        <v>0.02491764114594876</v>
+        <v>0.01094081453106472</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0.025x</t>
+          <t>0.011x</t>
         </is>
       </c>
       <c r="M39" t="n">
-        <v>0.02491764114594876</v>
+        <v>0.01094081453106472</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>0.025x</t>
+          <t>0.011x</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2558,49 +2558,49 @@
         <v>3</v>
       </c>
       <c r="E40" t="n">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="F40" t="n">
-        <v>0.001538019735305308</v>
+        <v>0.0003051989334171198</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>0.003843021418339992</v>
+        <v>0.001441114284775114</v>
       </c>
       <c r="I40" t="n">
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>0.02492163009404389</v>
+        <v>0.01373626373626374</v>
       </c>
       <c r="K40" t="n">
-        <v>0.5188086770309651</v>
+        <v>0.3942553618724525</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0.519x</t>
+          <t>0.394x</t>
         </is>
       </c>
       <c r="M40" t="n">
-        <v>0.01292748843766202</v>
+        <v>0.004313474792124307</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>0.013x</t>
+          <t>0.004x</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2612,49 +2612,49 @@
         <v>4</v>
       </c>
       <c r="E41" t="n">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="F41" t="n">
-        <v>0.001486461098652004</v>
+        <v>0.0003679439371722536</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>1.71860818924986e-05</v>
       </c>
       <c r="H41" t="n">
-        <v>0.004135700372420237</v>
+        <v>0.001476555200658624</v>
       </c>
       <c r="I41" t="n">
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>0.02492163009404389</v>
+        <v>0.01373626373626374</v>
       </c>
       <c r="K41" t="n">
-        <v>0.9664772593811553</v>
+        <v>1.205587231425148</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0.966x</t>
+          <t>1.206x</t>
         </is>
       </c>
       <c r="M41" t="n">
-        <v>0.01249412359591316</v>
+        <v>0.00520027013245931</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>0.012x</t>
+          <t>0.005x</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2669,46 +2669,46 @@
         <v>351</v>
       </c>
       <c r="F42" t="n">
-        <v>0.0008175586644413006</v>
+        <v>0.000179303612948414</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>0.003130494385334906</v>
+        <v>0.001045401853743629</v>
       </c>
       <c r="I42" t="n">
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>0.02492163009404389</v>
+        <v>0.01373626373626374</v>
       </c>
       <c r="K42" t="n">
-        <v>0.5500034041810464</v>
+        <v>0.4873123180841344</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0.550x</t>
+          <t>0.487x</t>
         </is>
       </c>
       <c r="M42" t="n">
-        <v>0.006871810510010975</v>
+        <v>0.002534155692912435</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>0.007x</t>
+          <t>0.003x</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2723,22 +2723,22 @@
         <v>2</v>
       </c>
       <c r="F43" t="n">
-        <v>1.825348372995303e-08</v>
+        <v>3.112614202830989e-08</v>
       </c>
       <c r="G43" t="n">
-        <v>1.825348372995303e-08</v>
+        <v>3.112614202830989e-08</v>
       </c>
       <c r="H43" t="n">
-        <v>7.708653197898958e-10</v>
+        <v>9.78051048024283e-09</v>
       </c>
       <c r="I43" t="n">
-        <v>1.770839963494805e-08</v>
+        <v>2.421027674426409e-08</v>
       </c>
       <c r="J43" t="n">
-        <v>1.8798567824958e-08</v>
+        <v>3.804200731235569e-08</v>
       </c>
       <c r="K43" t="n">
-        <v>2.232681827478032e-05</v>
+        <v>0.0001735946170658866</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="M43" t="n">
-        <v>1.534256644757405e-07</v>
+        <v>4.399157870964709e-07</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2777,19 +2777,19 @@
         <v>27</v>
       </c>
       <c r="F44" t="n">
-        <v>0.07013612366937573</v>
+        <v>0.08565092074072454</v>
       </c>
       <c r="G44" t="n">
-        <v>0.02400328046277493</v>
+        <v>0.03130113835245316</v>
       </c>
       <c r="H44" t="n">
-        <v>0.1390666291937573</v>
+        <v>0.160737741723825</v>
       </c>
       <c r="I44" t="n">
-        <v>0.0008048289738430583</v>
+        <v>0.002012072434607646</v>
       </c>
       <c r="J44" t="n">
-        <v>0.6783511846802986</v>
+        <v>0.7838364167478091</v>
       </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2829,34 +2829,34 @@
         <v>36</v>
       </c>
       <c r="F45" t="n">
-        <v>0.0005932209720691081</v>
+        <v>0.00712907591715185</v>
       </c>
       <c r="G45" t="n">
-        <v>4.67032399052543e-06</v>
+        <v>0.001094615536981008</v>
       </c>
       <c r="H45" t="n">
-        <v>0.002223799704063026</v>
+        <v>0.01887715056742475</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>0.01316391941391941</v>
+        <v>0.1025641025641026</v>
       </c>
       <c r="K45" t="n">
-        <v>0.008458137419535383</v>
+        <v>0.08323408383118734</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0.008x</t>
+          <t>0.083x</t>
         </is>
       </c>
       <c r="M45" t="n">
-        <v>0.008458137419535383</v>
+        <v>0.08323408383118734</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>0.008x</t>
+          <t>0.083x</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2883,34 +2883,34 @@
         <v>135</v>
       </c>
       <c r="F46" t="n">
-        <v>0.0001944774806201413</v>
+        <v>0.002415420459527441</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>0.0001757385769924955</v>
       </c>
       <c r="H46" t="n">
-        <v>0.001174650091758918</v>
+        <v>0.01027701012555062</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>0.01316391941391941</v>
+        <v>0.1025641025641026</v>
       </c>
       <c r="K46" t="n">
-        <v>0.3278331174668676</v>
+        <v>0.3388125596637537</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>0.328x</t>
+          <t>0.339x</t>
         </is>
       </c>
       <c r="M46" t="n">
-        <v>0.002772857558209452</v>
+        <v>0.02820075299411205</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>0.003x</t>
+          <t>0.028x</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2937,34 +2937,34 @@
         <v>171</v>
       </c>
       <c r="F47" t="n">
-        <v>0.0002510839789417186</v>
+        <v>0.002693106987006515</v>
       </c>
       <c r="G47" t="n">
-        <v>5.390883784482563e-06</v>
+        <v>0.0004018576933695114</v>
       </c>
       <c r="H47" t="n">
-        <v>0.001255439939709751</v>
+        <v>0.009552684334011262</v>
       </c>
       <c r="I47" t="n">
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>0.01316391941391941</v>
+        <v>0.1025641025641026</v>
       </c>
       <c r="K47" t="n">
-        <v>1.291069681389706</v>
+        <v>1.11496405372562</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>1.291x</t>
+          <t>1.115x</t>
         </is>
       </c>
       <c r="M47" t="n">
-        <v>0.003579952324216515</v>
+        <v>0.03144282587643008</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>0.004x</t>
+          <t>0.031x</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2991,34 +2991,34 @@
         <v>351</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0001223229640998116</v>
+        <v>0.001357784231723905</v>
       </c>
       <c r="G48" t="n">
-        <v>0</v>
+        <v>0.0001018507740658829</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0008839366586142033</v>
+        <v>0.006784993903677931</v>
       </c>
       <c r="I48" t="n">
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>0.01316391941391941</v>
+        <v>0.1025641025641026</v>
       </c>
       <c r="K48" t="n">
-        <v>0.4871794871794873</v>
+        <v>0.5041701790069361</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>0.487x</t>
+          <t>0.504x</t>
         </is>
       </c>
       <c r="M48" t="n">
-        <v>0.001744079337438815</v>
+        <v>0.01585253515060368</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>0.002x</t>
+          <t>0.016x</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>FullChain</t>
+          <t>CDR3a</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3045,46 +3045,46 @@
         <v>2</v>
       </c>
       <c r="F49" t="n">
-        <v>2.620715192312672e-08</v>
+        <v>0.0001298955201225842</v>
       </c>
       <c r="G49" t="n">
-        <v>2.620715192312672e-08</v>
+        <v>0.0001298955201225842</v>
       </c>
       <c r="H49" t="n">
-        <v>1.047732010961185e-08</v>
+        <v>5.959042875484255e-05</v>
       </c>
       <c r="I49" t="n">
-        <v>1.8798567824958e-08</v>
+        <v>8.775872385622115e-05</v>
       </c>
       <c r="J49" t="n">
-        <v>3.361573602129544e-08</v>
+        <v>0.0001720323163889472</v>
       </c>
       <c r="K49" t="n">
-        <v>0.0002142455598258927</v>
+        <v>0.09566727694109604</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>0.000x</t>
+          <t>0.096x</t>
         </is>
       </c>
       <c r="M49" t="n">
-        <v>3.73661254030351e-07</v>
+        <v>0.001516568870471261</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>0.000x</t>
+          <t>0.002x</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>FullAlpha</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3099,19 +3099,19 @@
         <v>27</v>
       </c>
       <c r="F50" t="n">
-        <v>0.1428016801844224</v>
+        <v>0.08714533050974928</v>
       </c>
       <c r="G50" t="n">
-        <v>0.1301775147928994</v>
+        <v>0.03391075472853033</v>
       </c>
       <c r="H50" t="n">
-        <v>0.09170777419687813</v>
+        <v>0.1486791053449375</v>
       </c>
       <c r="I50" t="n">
-        <v>0.0264367816091954</v>
+        <v>0.0008048289738430583</v>
       </c>
       <c r="J50" t="n">
-        <v>0.3883058470764618</v>
+        <v>0.6994482310938007</v>
       </c>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
@@ -3131,12 +3131,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>FullAlpha</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3148,49 +3148,49 @@
         <v>2</v>
       </c>
       <c r="E51" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="F51" t="n">
-        <v>0.01685383548180843</v>
+        <v>0.004776063527785849</v>
       </c>
       <c r="G51" t="n">
-        <v>0.005390588934741554</v>
+        <v>0.0004292298818519529</v>
       </c>
       <c r="H51" t="n">
-        <v>0.02684572963874532</v>
+        <v>0.01440360389873472</v>
       </c>
       <c r="I51" t="n">
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>0.1298374481398354</v>
+        <v>0.06818181818181818</v>
       </c>
       <c r="K51" t="n">
-        <v>0.118022669341442</v>
+        <v>0.05480573083891778</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>0.118x</t>
+          <t>0.055x</t>
         </is>
       </c>
       <c r="M51" t="n">
-        <v>0.118022669341442</v>
+        <v>0.05480573083891778</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>0.118x</t>
+          <t>0.055x</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>FullAlpha</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3202,49 +3202,49 @@
         <v>3</v>
       </c>
       <c r="E52" t="n">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="F52" t="n">
-        <v>0.008934128277050243</v>
+        <v>0.003347140588238225</v>
       </c>
       <c r="G52" t="n">
-        <v>0.001218086055301858</v>
+        <v>0.0002648893113267449</v>
       </c>
       <c r="H52" t="n">
-        <v>0.02053450368074804</v>
+        <v>0.009228045923148144</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>0.1298374481398354</v>
+        <v>0.06818181818181818</v>
       </c>
       <c r="K52" t="n">
-        <v>0.5300946651991172</v>
+        <v>0.7008157594147281</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>0.530x</t>
+          <t>0.701x</t>
         </is>
       </c>
       <c r="M52" t="n">
-        <v>0.0625631873904578</v>
+        <v>0.03840871987815535</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>0.063x</t>
+          <t>0.038x</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>FullAlpha</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3256,49 +3256,49 @@
         <v>4</v>
       </c>
       <c r="E53" t="n">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="F53" t="n">
-        <v>0.006610525272294024</v>
+        <v>0.002334549589353883</v>
       </c>
       <c r="G53" t="n">
-        <v>0.0009613073780341264</v>
+        <v>0.000230859637340497</v>
       </c>
       <c r="H53" t="n">
-        <v>0.0164585619713131</v>
+        <v>0.007912764679275474</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>0.1298374481398354</v>
+        <v>0.06818181818181818</v>
       </c>
       <c r="K53" t="n">
-        <v>0.7399183297238937</v>
+        <v>0.6974758089210346</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>0.740x</t>
+          <t>0.697x</t>
         </is>
       </c>
       <c r="M53" t="n">
-        <v>0.0462916491161505</v>
+        <v>0.02678915296663782</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>0.046x</t>
+          <t>0.027x</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>FullAlpha</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3313,46 +3313,46 @@
         <v>351</v>
       </c>
       <c r="F54" t="n">
-        <v>0.003841069855168812</v>
+        <v>0.001563182077865423</v>
       </c>
       <c r="G54" t="n">
-        <v>0.0001560695445890689</v>
+        <v>0.0001166393293238564</v>
       </c>
       <c r="H54" t="n">
-        <v>0.01245847079403397</v>
+        <v>0.006004885927801725</v>
       </c>
       <c r="I54" t="n">
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>0.1298374481398354</v>
+        <v>0.06818181818181818</v>
       </c>
       <c r="K54" t="n">
-        <v>0.5810536526147886</v>
+        <v>0.669586152718244</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>0.581x</t>
+          <t>0.670x</t>
         </is>
       </c>
       <c r="M54" t="n">
-        <v>0.0268979318045014</v>
+        <v>0.01793764586951155</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>0.027x</t>
+          <t>0.018x</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>FullAlpha</t>
+          <t>CDR3b</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3367,30 +3367,30 @@
         <v>2</v>
       </c>
       <c r="F55" t="n">
-        <v>2.452959985183437e-05</v>
+        <v>1.584501002217626e-05</v>
       </c>
       <c r="G55" t="n">
-        <v>2.452959985183437e-05</v>
+        <v>1.584501002217626e-05</v>
       </c>
       <c r="H55" t="n">
-        <v>1.282136692836654e-05</v>
+        <v>1.657007775314753e-06</v>
       </c>
       <c r="I55" t="n">
-        <v>1.546352435270545e-05</v>
+        <v>1.467332858777236e-05</v>
       </c>
       <c r="J55" t="n">
-        <v>3.359567535096329e-05</v>
+        <v>1.701669145658016e-05</v>
       </c>
       <c r="K55" t="n">
-        <v>0.006386137398367183</v>
+        <v>0.0101363815812251</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>0.006x</t>
+          <t>0.010x</t>
         </is>
       </c>
       <c r="M55" t="n">
-        <v>0.0001717738882354564</v>
+        <v>0.0001818228232022554</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3743,19 +3743,19 @@
         <v>27</v>
       </c>
       <c r="F62" t="n">
-        <v>0.1540154431948367</v>
+        <v>0.08678965795430232</v>
       </c>
       <c r="G62" t="n">
-        <v>0.1158402203856749</v>
+        <v>0.03382300126592495</v>
       </c>
       <c r="H62" t="n">
-        <v>0.1055437468616878</v>
+        <v>0.1484144060676106</v>
       </c>
       <c r="I62" t="n">
-        <v>0.01686702078091511</v>
+        <v>0.0008048289738430583</v>
       </c>
       <c r="J62" t="n">
-        <v>0.4321200621010868</v>
+        <v>0.6994482310938007</v>
       </c>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
@@ -3775,7 +3775,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3792,44 +3792,44 @@
         <v>2</v>
       </c>
       <c r="E63" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="F63" t="n">
-        <v>0.01782030571915158</v>
+        <v>0.00315228236576409</v>
       </c>
       <c r="G63" t="n">
-        <v>0.006677088898509607</v>
+        <v>0.000302155638177779</v>
       </c>
       <c r="H63" t="n">
-        <v>0.04924877471640624</v>
+        <v>0.01157355516675025</v>
       </c>
       <c r="I63" t="n">
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>0.3612068965517241</v>
+        <v>0.06818181818181818</v>
       </c>
       <c r="K63" t="n">
-        <v>0.1157046679832493</v>
+        <v>0.03632094468472122</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>0.116x</t>
+          <t>0.036x</t>
         </is>
       </c>
       <c r="M63" t="n">
-        <v>0.1157046679832493</v>
+        <v>0.03632094468472122</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>0.116x</t>
+          <t>0.036x</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3846,44 +3846,44 @@
         <v>3</v>
       </c>
       <c r="E64" t="n">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="F64" t="n">
-        <v>0.01253593281963678</v>
+        <v>0.001296231924362134</v>
       </c>
       <c r="G64" t="n">
-        <v>0.00271411335360849</v>
+        <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>0.04210089482392654</v>
+        <v>0.006352531662463185</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>0.3612068965517241</v>
+        <v>0.06818181818181818</v>
       </c>
       <c r="K64" t="n">
-        <v>0.7034633982830242</v>
+        <v>0.4112042558243152</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>0.703x</t>
+          <t>0.411x</t>
         </is>
       </c>
       <c r="M64" t="n">
-        <v>0.0813939989367056</v>
+        <v>0.01493532702991691</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>0.081x</t>
+          <t>0.015x</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3900,44 +3900,44 @@
         <v>4</v>
       </c>
       <c r="E65" t="n">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="F65" t="n">
-        <v>0.00705422976093418</v>
+        <v>0.001021445758264269</v>
       </c>
       <c r="G65" t="n">
-        <v>0.0004251700680272109</v>
+        <v>3.510272169380735e-05</v>
       </c>
       <c r="H65" t="n">
-        <v>0.02797947491014535</v>
+        <v>0.005539185805200156</v>
       </c>
       <c r="I65" t="n">
         <v>0</v>
       </c>
       <c r="J65" t="n">
-        <v>0.3612068965517241</v>
+        <v>0.06818181818181818</v>
       </c>
       <c r="K65" t="n">
-        <v>0.5627207693618265</v>
+        <v>0.7880115734434748</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>0.563x</t>
+          <t>0.788x</t>
         </is>
       </c>
       <c r="M65" t="n">
-        <v>0.04580209370309865</v>
+        <v>0.01176921055273768</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>0.046x</t>
+          <t>0.012x</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3957,41 +3957,41 @@
         <v>351</v>
       </c>
       <c r="F66" t="n">
-        <v>0.005335151368539006</v>
+        <v>0.0006672592877457144</v>
       </c>
       <c r="G66" t="n">
-        <v>0.0002297794117647059</v>
+        <v>0</v>
       </c>
       <c r="H66" t="n">
-        <v>0.02449839159150042</v>
+        <v>0.004079177238988301</v>
       </c>
       <c r="I66" t="n">
         <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>0.3612068965517241</v>
+        <v>0.06818181818181818</v>
       </c>
       <c r="K66" t="n">
-        <v>0.7563053018324826</v>
+        <v>0.6532498493895365</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>0.756x</t>
+          <t>0.653x</t>
         </is>
       </c>
       <c r="M66" t="n">
-        <v>0.03464036630268168</v>
+        <v>0.007688235021009633</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>0.035x</t>
+          <t>0.008x</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Kb</t>
+          <t>Kd</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4011,30 +4011,30 @@
         <v>2</v>
       </c>
       <c r="F67" t="n">
-        <v>8.290285626479562e-06</v>
+        <v>6.886124960477805e-06</v>
       </c>
       <c r="G67" t="n">
-        <v>8.290285626479562e-06</v>
+        <v>6.886124960477805e-06</v>
       </c>
       <c r="H67" t="n">
-        <v>1.770770382762725e-06</v>
+        <v>3.756553440373247e-06</v>
       </c>
       <c r="I67" t="n">
-        <v>7.038161880903741e-06</v>
+        <v>4.229840548900228e-06</v>
       </c>
       <c r="J67" t="n">
         <v>9.542409372055383e-06</v>
       </c>
       <c r="K67" t="n">
-        <v>0.001553898859433823</v>
+        <v>0.01032001365427533</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>0.002x</t>
+          <t>0.010x</t>
         </is>
       </c>
       <c r="M67" t="n">
-        <v>5.382762568810689e-05</v>
+        <v>7.934269039409721e-05</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
@@ -4050,7 +4050,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>FullBeta</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -4065,19 +4065,19 @@
         <v>27</v>
       </c>
       <c r="F68" t="n">
-        <v>0.08678965795430232</v>
+        <v>0.07013612366937573</v>
       </c>
       <c r="G68" t="n">
-        <v>0.03382300126592495</v>
+        <v>0.02400328046277493</v>
       </c>
       <c r="H68" t="n">
-        <v>0.1484144060676106</v>
+        <v>0.1390666291937573</v>
       </c>
       <c r="I68" t="n">
         <v>0.0008048289738430583</v>
       </c>
       <c r="J68" t="n">
-        <v>0.6994482310938007</v>
+        <v>0.6783511846802986</v>
       </c>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>FullBeta</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -4117,34 +4117,34 @@
         <v>36</v>
       </c>
       <c r="F69" t="n">
-        <v>0.00315228236576409</v>
+        <v>0.0005932209720691081</v>
       </c>
       <c r="G69" t="n">
-        <v>0.000302155638177779</v>
+        <v>4.67032399052543e-06</v>
       </c>
       <c r="H69" t="n">
-        <v>0.01157355516675025</v>
+        <v>0.002223799704063026</v>
       </c>
       <c r="I69" t="n">
         <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>0.06818181818181818</v>
+        <v>0.01316391941391941</v>
       </c>
       <c r="K69" t="n">
-        <v>0.03632094468472122</v>
+        <v>0.008458137419535383</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>0.036x</t>
+          <t>0.008x</t>
         </is>
       </c>
       <c r="M69" t="n">
-        <v>0.03632094468472122</v>
+        <v>0.008458137419535383</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>0.036x</t>
+          <t>0.008x</t>
         </is>
       </c>
     </row>
@@ -4156,7 +4156,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>FullBeta</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -4171,34 +4171,34 @@
         <v>135</v>
       </c>
       <c r="F70" t="n">
-        <v>0.001296231924362134</v>
+        <v>0.0001944774806201413</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
       </c>
       <c r="H70" t="n">
-        <v>0.006352531662463185</v>
+        <v>0.001174650091758918</v>
       </c>
       <c r="I70" t="n">
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>0.06818181818181818</v>
+        <v>0.01316391941391941</v>
       </c>
       <c r="K70" t="n">
-        <v>0.4112042558243152</v>
+        <v>0.3278331174668676</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>0.411x</t>
+          <t>0.328x</t>
         </is>
       </c>
       <c r="M70" t="n">
-        <v>0.01493532702991691</v>
+        <v>0.002772857558209452</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>0.015x</t>
+          <t>0.003x</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>FullBeta</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -4225,34 +4225,34 @@
         <v>171</v>
       </c>
       <c r="F71" t="n">
-        <v>0.001021445758264269</v>
+        <v>0.0002510839789417186</v>
       </c>
       <c r="G71" t="n">
-        <v>3.510272169380735e-05</v>
+        <v>5.390883784482563e-06</v>
       </c>
       <c r="H71" t="n">
-        <v>0.005539185805200156</v>
+        <v>0.001255439939709751</v>
       </c>
       <c r="I71" t="n">
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>0.06818181818181818</v>
+        <v>0.01316391941391941</v>
       </c>
       <c r="K71" t="n">
-        <v>0.7880115734434748</v>
+        <v>1.291069681389706</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>0.788x</t>
+          <t>1.291x</t>
         </is>
       </c>
       <c r="M71" t="n">
-        <v>0.01176921055273768</v>
+        <v>0.003579952324216515</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>0.012x</t>
+          <t>0.004x</t>
         </is>
       </c>
     </row>
@@ -4264,7 +4264,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>FullBeta</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -4279,34 +4279,34 @@
         <v>351</v>
       </c>
       <c r="F72" t="n">
-        <v>0.0006672592877457144</v>
+        <v>0.0001223229640998116</v>
       </c>
       <c r="G72" t="n">
         <v>0</v>
       </c>
       <c r="H72" t="n">
-        <v>0.004079177238988301</v>
+        <v>0.0008839366586142033</v>
       </c>
       <c r="I72" t="n">
         <v>0</v>
       </c>
       <c r="J72" t="n">
-        <v>0.06818181818181818</v>
+        <v>0.01316391941391941</v>
       </c>
       <c r="K72" t="n">
-        <v>0.6532498493895365</v>
+        <v>0.4871794871794873</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>0.653x</t>
+          <t>0.487x</t>
         </is>
       </c>
       <c r="M72" t="n">
-        <v>0.007688235021009633</v>
+        <v>0.001744079337438815</v>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>0.008x</t>
+          <t>0.002x</t>
         </is>
       </c>
     </row>
@@ -4318,7 +4318,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>FullBeta</t>
+          <t>FullChain</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -4333,30 +4333,30 @@
         <v>2</v>
       </c>
       <c r="F73" t="n">
-        <v>6.886124960477805e-06</v>
+        <v>2.620715192312672e-08</v>
       </c>
       <c r="G73" t="n">
-        <v>6.886124960477805e-06</v>
+        <v>2.620715192312672e-08</v>
       </c>
       <c r="H73" t="n">
-        <v>3.756553440373247e-06</v>
+        <v>1.047732010961185e-08</v>
       </c>
       <c r="I73" t="n">
-        <v>4.229840548900228e-06</v>
+        <v>1.8798567824958e-08</v>
       </c>
       <c r="J73" t="n">
-        <v>9.542409372055383e-06</v>
+        <v>3.361573602129544e-08</v>
       </c>
       <c r="K73" t="n">
-        <v>0.01032001365427533</v>
+        <v>0.0002142455598258927</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>0.010x</t>
+          <t>0.000x</t>
         </is>
       </c>
       <c r="M73" t="n">
-        <v>7.934269039409721e-05</v>
+        <v>3.73661254030351e-07</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
added same strain, different mhc and same mhc, different strain points to the singleset plots also introduced de-duplication also recreated pc plots from mayer and callan but for this data
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/pc_summary_statistics.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/pc_summary_statistics.xlsx
@@ -513,7 +513,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -565,7 +565,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -619,7 +619,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -673,7 +673,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -727,7 +727,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -781,32 +781,32 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>2.185434755743738e-08</v>
+        <v>1.114644974255831e-08</v>
       </c>
       <c r="G7" t="n">
-        <v>2.185434755743738e-08</v>
+        <v>1.018776111298458e-08</v>
       </c>
       <c r="H7" t="n">
-        <v>3.331787008000945e-09</v>
+        <v>1.251827680778248e-08</v>
       </c>
       <c r="I7" t="n">
-        <v>1.949841837061067e-08</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
         <v>2.421027674426409e-08</v>
       </c>
       <c r="K7" t="n">
-        <v>1.850980633244098e-05</v>
+        <v>9.440621619419036e-06</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>1.771073027116946e-07</v>
+        <v>9.033066045680881e-08</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -835,7 +835,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -887,7 +887,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -941,7 +941,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -995,7 +995,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1103,23 +1103,23 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D13" t="n">
         <v>6</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0001169694818177544</v>
+        <v>9.422539473744542e-05</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0001169694818177544</v>
+        <v>7.148130765713644e-05</v>
       </c>
       <c r="H13" t="n">
-        <v>7.787060743328694e-05</v>
+        <v>5.225266420089913e-05</v>
       </c>
       <c r="I13" t="n">
         <v>6.190664724656162e-05</v>
@@ -1128,15 +1128,15 @@
         <v>0.0001720323163889472</v>
       </c>
       <c r="K13" t="n">
-        <v>0.01782302565926867</v>
+        <v>0.01435743411069212</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0.018x</t>
+          <t>0.014x</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>0.0007619116498710066</v>
+        <v>0.0006137620244912202</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1425,32 +1425,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>6</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>1.507953647152783e-05</v>
+        <v>1.907483524663574e-05</v>
       </c>
       <c r="G19" t="n">
         <v>1.507953647152783e-05</v>
       </c>
       <c r="H19" t="n">
-        <v>2.739550852279648e-06</v>
+        <v>1.124055681267341e-05</v>
       </c>
       <c r="I19" t="n">
-        <v>1.314238148647551e-05</v>
+        <v>1.066659492406927e-05</v>
       </c>
       <c r="J19" t="n">
-        <v>1.701669145658016e-05</v>
+        <v>3.547367311941806e-05</v>
       </c>
       <c r="K19" t="n">
-        <v>0.00271480446225338</v>
+        <v>0.003434087509393322</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>9.769106386055242e-05</v>
+        <v>0.0001235741530734073</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1747,40 +1747,40 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D25" t="n">
         <v>6</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>2.452959985183437e-05</v>
+        <v>1.25055175293869e-05</v>
       </c>
       <c r="G25" t="n">
-        <v>2.452959985183437e-05</v>
+        <v>8.121415564095736e-06</v>
       </c>
       <c r="H25" t="n">
-        <v>1.282136692836654e-05</v>
+        <v>1.573614869912037e-05</v>
       </c>
       <c r="I25" t="n">
-        <v>1.546352435270545e-05</v>
+        <v>1.83563638392849e-07</v>
       </c>
       <c r="J25" t="n">
         <v>3.359567535096329e-05</v>
       </c>
       <c r="K25" t="n">
-        <v>0.006386137398367183</v>
+        <v>0.00325573811487927</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0.006x</t>
+          <t>0.003x</t>
         </is>
       </c>
       <c r="M25" t="n">
-        <v>0.0001717738882354564</v>
+        <v>8.757262178733856e-05</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -2069,40 +2069,40 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D31" t="n">
         <v>6</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F31" t="n">
-        <v>8.290285626479562e-06</v>
+        <v>5.227438658173412e-06</v>
       </c>
       <c r="G31" t="n">
-        <v>8.290285626479562e-06</v>
+        <v>5.614836265921813e-06</v>
       </c>
       <c r="H31" t="n">
-        <v>1.770770382762725e-06</v>
+        <v>4.036357883993514e-06</v>
       </c>
       <c r="I31" t="n">
-        <v>7.038161880903741e-06</v>
+        <v>1.376727287946367e-07</v>
       </c>
       <c r="J31" t="n">
         <v>9.542409372055383e-06</v>
       </c>
       <c r="K31" t="n">
-        <v>0.001553898859433823</v>
+        <v>0.000979810748950673</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0.002x</t>
+          <t>0.001x</t>
         </is>
       </c>
       <c r="M31" t="n">
-        <v>5.382762568810689e-05</v>
+        <v>3.394100325095619e-05</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2391,32 +2391,32 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D37" t="n">
         <v>6</v>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F37" t="n">
-        <v>1.825348372995303e-08</v>
+        <v>9.160476628644147e-09</v>
       </c>
       <c r="G37" t="n">
-        <v>1.825348372995303e-08</v>
+        <v>8.921669344809296e-09</v>
       </c>
       <c r="H37" t="n">
-        <v>7.708653197898958e-10</v>
+        <v>1.050927289259835e-08</v>
       </c>
       <c r="I37" t="n">
-        <v>1.770839963494805e-08</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
         <v>1.8798567824958e-08</v>
       </c>
       <c r="K37" t="n">
-        <v>2.232681827478032e-05</v>
+        <v>1.120467194229321e-05</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="M37" t="n">
-        <v>1.534256644757405e-07</v>
+        <v>7.699638241427554e-08</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2713,32 +2713,32 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D43" t="n">
         <v>6</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F43" t="n">
-        <v>3.112614202830989e-08</v>
+        <v>1.58745647897548e-08</v>
       </c>
       <c r="G43" t="n">
-        <v>3.112614202830989e-08</v>
+        <v>1.272812592333176e-08</v>
       </c>
       <c r="H43" t="n">
-        <v>9.78051048024283e-09</v>
+        <v>1.85011445167273e-08</v>
       </c>
       <c r="I43" t="n">
-        <v>2.421027674426409e-08</v>
+        <v>0</v>
       </c>
       <c r="J43" t="n">
         <v>3.804200731235569e-08</v>
       </c>
       <c r="K43" t="n">
-        <v>0.0001735946170658866</v>
+        <v>8.853455057998158e-05</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="M43" t="n">
-        <v>4.399157870964709e-07</v>
+        <v>2.243603353717043e-07</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -3035,44 +3035,44 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D49" t="n">
         <v>6</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0001298955201225842</v>
+        <v>0.000106612077437178</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0001298955201225842</v>
+        <v>8.877435989137968e-05</v>
       </c>
       <c r="H49" t="n">
-        <v>5.959042875484255e-05</v>
+        <v>4.398102768537776e-05</v>
       </c>
       <c r="I49" t="n">
-        <v>8.775872385622115e-05</v>
+        <v>7.68672735770055e-05</v>
       </c>
       <c r="J49" t="n">
         <v>0.0001720323163889472</v>
       </c>
       <c r="K49" t="n">
-        <v>0.09566727694109604</v>
+        <v>0.07851916007436499</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>0.096x</t>
+          <t>0.079x</t>
         </is>
       </c>
       <c r="M49" t="n">
-        <v>0.001516568870471261</v>
+        <v>0.001244727745074748</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>0.002x</t>
+          <t>0.001x</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -3141,7 +3141,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3357,40 +3357,40 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D55" t="n">
         <v>6</v>
       </c>
       <c r="E55" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F55" t="n">
-        <v>1.584501002217626e-05</v>
+        <v>1.940121805685643e-05</v>
       </c>
       <c r="G55" t="n">
         <v>1.584501002217626e-05</v>
       </c>
       <c r="H55" t="n">
-        <v>1.657007775314753e-06</v>
+        <v>1.10550895735411e-05</v>
       </c>
       <c r="I55" t="n">
-        <v>1.467332858777236e-05</v>
+        <v>1.044117906365516e-05</v>
       </c>
       <c r="J55" t="n">
-        <v>1.701669145658016e-05</v>
+        <v>3.547367311941806e-05</v>
       </c>
       <c r="K55" t="n">
-        <v>0.0101363815812251</v>
+        <v>0.01241136162675908</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>0.010x</t>
+          <t>0.012x</t>
         </is>
       </c>
       <c r="M55" t="n">
-        <v>0.0001818228232022554</v>
+        <v>0.0002226306096192491</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3679,40 +3679,40 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D61" t="n">
         <v>6</v>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F61" t="n">
-        <v>2.717182129218875e-05</v>
+        <v>1.703150230662194e-05</v>
       </c>
       <c r="G61" t="n">
-        <v>2.717182129218875e-05</v>
+        <v>1.717338511856581e-05</v>
       </c>
       <c r="H61" t="n">
-        <v>9.084701532624403e-06</v>
+        <v>1.395015414571385e-05</v>
       </c>
       <c r="I61" t="n">
-        <v>2.074796723341422e-05</v>
+        <v>1.83563638392849e-07</v>
       </c>
       <c r="J61" t="n">
         <v>3.359567535096329e-05</v>
       </c>
       <c r="K61" t="n">
-        <v>0.04430623918254412</v>
+        <v>0.02777148453615708</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>0.044x</t>
+          <t>0.028x</t>
         </is>
       </c>
       <c r="M61" t="n">
-        <v>0.0003267135659630848</v>
+        <v>0.0002047865247039806</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3893,7 +3893,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -4001,40 +4001,40 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D67" t="n">
         <v>6</v>
       </c>
       <c r="E67" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F67" t="n">
-        <v>6.886124960477805e-06</v>
+        <v>4.099187628115363e-06</v>
       </c>
       <c r="G67" t="n">
-        <v>6.886124960477805e-06</v>
+        <v>3.358334205805718e-06</v>
       </c>
       <c r="H67" t="n">
-        <v>3.756553440373247e-06</v>
+        <v>3.997459086721851e-06</v>
       </c>
       <c r="I67" t="n">
-        <v>4.229840548900228e-06</v>
+        <v>1.376727287946367e-07</v>
       </c>
       <c r="J67" t="n">
         <v>9.542409372055383e-06</v>
       </c>
       <c r="K67" t="n">
-        <v>0.01032001365427533</v>
+        <v>0.006143320450381683</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>0.010x</t>
+          <t>0.006x</t>
         </is>
       </c>
       <c r="M67" t="n">
-        <v>7.934269039409721e-05</v>
+        <v>4.723129143190913e-05</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>within epitope within mice</t>
+          <t>Single mouse</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>within strain &amp; epitope across mice</t>
+          <t>Same strain, same epitope</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>within epitope across strain</t>
+          <t>Same epitope, different strain</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -4215,7 +4215,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>within strain across epitope</t>
+          <t>Same strain, different epitope</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>across strain across epitope</t>
+          <t>Cross-strain baseline</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4323,32 +4323,32 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Pre-Immune Repertoires</t>
+          <t>Pre-Immune Repertoire</t>
         </is>
       </c>
       <c r="D73" t="n">
         <v>6</v>
       </c>
       <c r="E73" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F73" t="n">
-        <v>2.620715192312672e-08</v>
+        <v>1.314972318757815e-08</v>
       </c>
       <c r="G73" t="n">
-        <v>2.620715192312672e-08</v>
+        <v>9.491578364508586e-09</v>
       </c>
       <c r="H73" t="n">
-        <v>1.047732010961185e-08</v>
+        <v>1.624578975146838e-08</v>
       </c>
       <c r="I73" t="n">
-        <v>1.8798567824958e-08</v>
+        <v>0</v>
       </c>
       <c r="J73" t="n">
         <v>3.361573602129544e-08</v>
       </c>
       <c r="K73" t="n">
-        <v>0.0002142455598258927</v>
+        <v>0.0001075000371708488</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -4356,7 +4356,7 @@
         </is>
       </c>
       <c r="M73" t="n">
-        <v>3.73661254030351e-07</v>
+        <v>1.87488593603582e-07</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>

</xml_diff>